<commit_message>
Include actual resource files and parsed layers
</commit_message>
<xml_diff>
--- a/outputs/01a12ec5-33b0-73d0-b60b-e9ed1659461e/CALE任务卡材料库.xlsx
+++ b/outputs/01a12ec5-33b0-73d0-b60b-e9ed1659461e/CALE任务卡材料库.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡片覆盖" sheetId="1" r:id="Rf9508360c319450f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料目录" sheetId="2" r:id="R6d0d5ff2b6d34cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输入缺口" sheetId="3" r:id="Rb231bbbe2c294fb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡片覆盖" sheetId="1" r:id="Rbd4d28a1b4404714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料目录" sheetId="2" r:id="R7d43020b786249bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输入缺口" sheetId="3" r:id="Rbb487941f4bc444a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -260,10 +260,10 @@
     <x:tableColumn id="7" name="材料角色"/>
     <x:tableColumn id="8" name="取得状态"/>
     <x:tableColumn id="9" name="质量记录"/>
-    <x:tableColumn id="10" name="PDF页数"/>
+    <x:tableColumn id="10" name="入库PDF页数"/>
     <x:tableColumn id="11" name="大小 MB"/>
     <x:tableColumn id="12" name="来源"/>
-    <x:tableColumn id="13" name="原件"/>
+    <x:tableColumn id="13" name="仓库文件"/>
     <x:tableColumn id="14" name="待处理事项"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -858,7 +858,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb321a29083294017"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd8ab0d86c7341cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -922,7 +922,7 @@
     </row>
     <row r="3" ht="17.25" customHeight="1">
       <c r="A3" s="2" t="str">
-        <v>41 条记录：39 份本地原件、2 条版权受限的规则链接。</v>
+        <v>39 份仓库材料：38 份完整原件、1 份业务副本；另有 2 条受限链接。</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1011,7 +1011,7 @@
         <v>质量记录</v>
       </c>
       <c r="J6" s="15" t="str">
-        <v>PDF页数</v>
+        <v>入库PDF页数</v>
       </c>
       <c r="K6" s="15" t="str">
         <v>大小 MB</v>
@@ -1020,7 +1020,7 @@
         <v>来源</v>
       </c>
       <c r="M6" s="15" t="str">
-        <v>原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N6" s="16" t="str">
         <v>待处理事项</v>
@@ -1064,7 +1064,7 @@
         <v>官方原件</v>
       </c>
       <c r="M7" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N7" s="19" t="str"/>
     </row>
@@ -1106,7 +1106,7 @@
         <v>官方原件</v>
       </c>
       <c r="M8" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N8" s="20" t="str"/>
     </row>
@@ -1148,7 +1148,7 @@
         <v>官方原件</v>
       </c>
       <c r="M9" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N9" s="19" t="str"/>
     </row>
@@ -1190,7 +1190,7 @@
         <v>官方原件</v>
       </c>
       <c r="M10" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N10" s="20" t="str"/>
     </row>
@@ -1234,7 +1234,7 @@
         <v>官方原件</v>
       </c>
       <c r="M11" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N11" s="19" t="str"/>
     </row>
@@ -1277,7 +1277,7 @@
         <v>官方原件</v>
       </c>
       <c r="M12" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N12" s="20" t="str"/>
     </row>
@@ -1319,7 +1319,7 @@
         <v>官方原件</v>
       </c>
       <c r="M13" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N13" s="19" t="str"/>
     </row>
@@ -1361,7 +1361,7 @@
         <v>官方原件</v>
       </c>
       <c r="M14" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N14" s="20" t="str">
         <v>全扫描PDF；已保留逐页OCR及置信度；任何用于评分的关键数值/条款均需回看原页</v>
@@ -1405,7 +1405,7 @@
         <v>官方原件</v>
       </c>
       <c r="M15" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N15" s="19" t="str"/>
     </row>
@@ -1447,7 +1447,7 @@
         <v>官方原件</v>
       </c>
       <c r="M16" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N16" s="20" t="str"/>
     </row>
@@ -1489,7 +1489,7 @@
         <v>官方原件</v>
       </c>
       <c r="M17" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N17" s="19" t="str"/>
     </row>
@@ -1531,7 +1531,7 @@
         <v>官方原件</v>
       </c>
       <c r="M18" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N18" s="20" t="str"/>
     </row>
@@ -1573,7 +1573,7 @@
         <v>官方原件</v>
       </c>
       <c r="M19" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N19" s="19" t="str">
         <v>全扫描PDF；已保留逐页OCR及置信度；任何用于评分的关键数值/条款均需回看原页</v>
@@ -1617,7 +1617,7 @@
         <v>官方原件</v>
       </c>
       <c r="M20" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N20" s="20" t="str"/>
     </row>
@@ -1659,7 +1659,7 @@
         <v>官方原件</v>
       </c>
       <c r="M21" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N21" s="19" t="str"/>
     </row>
@@ -1701,7 +1701,7 @@
         <v>官方原件</v>
       </c>
       <c r="M22" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N22" s="20" t="str"/>
     </row>
@@ -1743,7 +1743,7 @@
         <v>官方原件</v>
       </c>
       <c r="M23" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N23" s="19" t="str"/>
     </row>
@@ -1786,7 +1786,7 @@
         <v>官方原件</v>
       </c>
       <c r="M24" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N24" s="20" t="str">
         <v>更正后报表封面沿用2026-04-29，实际更正版披露2026-08-06；按版本关系记录</v>
@@ -1822,16 +1822,16 @@
         <v>原件通过，需处理问题</v>
       </c>
       <c r="J25" s="25" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K25" s="27" t="n">
-        <v>2.1991939544677734</v>
+        <v>1.2456979751586914</v>
       </c>
       <c r="L25" s="29" t="str">
         <v>官方原件</v>
       </c>
       <c r="M25" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N25" s="19" t="str">
         <v>全扫描PDF；正文页1-6保留OCR；证照/个人信息附页7-10不进入派生层或任务输入
@@ -1877,7 +1877,7 @@
         <v>官方原件</v>
       </c>
       <c r="M26" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N26" s="20" t="str"/>
     </row>
@@ -1919,7 +1919,7 @@
         <v>官方原件</v>
       </c>
       <c r="M27" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N27" s="19" t="str">
         <v>公司对案情及诉请的披露不是法院查明或原始证据；旧案已裁判结论不作新案事前输入</v>
@@ -1963,7 +1963,7 @@
         <v>官方原件</v>
       </c>
       <c r="M28" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N28" s="20" t="str"/>
     </row>
@@ -2007,7 +2007,7 @@
         <v>官方原件</v>
       </c>
       <c r="M29" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N29" s="19" t="str">
         <v>2026半年报未经审计，不能标为审计报表；币种人民币、单位元与其他披露万元分开</v>
@@ -2051,7 +2051,7 @@
         <v>官方原件</v>
       </c>
       <c r="M30" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N30" s="20" t="str">
         <v>兑付公告说明计划/安排，不能据此判定资金已到账</v>
@@ -2093,7 +2093,7 @@
         <v>官方原件</v>
       </c>
       <c r="M31" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N31" s="19" t="str"/>
     </row>
@@ -2135,7 +2135,7 @@
         <v>官方原件</v>
       </c>
       <c r="M32" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N32" s="20" t="str"/>
     </row>
@@ -2175,7 +2175,7 @@
         <v>官方原件</v>
       </c>
       <c r="M33" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N33" s="19" t="str"/>
     </row>
@@ -2215,7 +2215,7 @@
         <v>官方原件</v>
       </c>
       <c r="M34" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N34" s="20" t="str"/>
     </row>
@@ -2255,7 +2255,7 @@
         <v>官方原件</v>
       </c>
       <c r="M35" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N35" s="19" t="str"/>
     </row>
@@ -2295,7 +2295,7 @@
         <v>官方原件</v>
       </c>
       <c r="M36" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N36" s="20" t="str">
         <v>原生工作簿存在打印区域之外大量重复表头、合并区域及空白Sheet2；可用区域按官方打印设置A2:Q18（含A1附件标题）核对
@@ -2338,7 +2338,7 @@
         <v>官方原件</v>
       </c>
       <c r="M37" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N37" s="19" t="str">
         <v>保留未签模板与CZ2026-xxxx占位；不得冒充签署稿
@@ -2381,7 +2381,7 @@
         <v>官方原件</v>
       </c>
       <c r="M38" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N38" s="20" t="str"/>
     </row>
@@ -2421,7 +2421,7 @@
         <v>官方原件</v>
       </c>
       <c r="M39" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N39" s="19" t="str">
         <v>ZIP仅作原始容器，内部PDF/Word与独立章节不作为独立来源重复计数</v>
@@ -2541,7 +2541,7 @@
         <v>官方原件</v>
       </c>
       <c r="M42" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N42" s="20" t="str">
         <v>前24页为扫描内容；OCR不作为数值金标准</v>
@@ -2585,7 +2585,7 @@
         <v>官方原件</v>
       </c>
       <c r="M43" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N43" s="19" t="str"/>
     </row>
@@ -2627,7 +2627,7 @@
         <v>官方原件</v>
       </c>
       <c r="M44" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N44" s="20" t="str"/>
     </row>
@@ -2669,7 +2669,7 @@
         <v>官方原件</v>
       </c>
       <c r="M45" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N45" s="19" t="str"/>
     </row>
@@ -2711,7 +2711,7 @@
         <v>官方原件</v>
       </c>
       <c r="M46" s="30" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N46" s="20" t="str"/>
     </row>
@@ -2753,7 +2753,7 @@
         <v>官方原件</v>
       </c>
       <c r="M47" s="29" t="str">
-        <v>本地原件</v>
+        <v>仓库文件</v>
       </c>
       <c r="N47" s="19" t="str"/>
     </row>
@@ -2848,7 +2848,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Rca6961ab0d204b00"/>
+    <tablePart r:id="Rff9763263c194dc4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3793,7 +3793,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc43b9288f6d641ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bd71ecbdfbe4b18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>